<commit_message>
General updates to PHA4GE to ODM v2 ID generation
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
+++ b/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/pha4ge-to-v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93C10C96-1782-0840-A169-103D31039A8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{290A3B4D-8B58-0043-927B-63B4BFB46AB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{7D7FC1CC-FEF0-9E4D-91AE-A58F443803E1}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>sites</t>
   </si>
@@ -98,6 +98,15 @@
   </si>
   <si>
     <t>dat.samples.get_first_linked_value("sampleID", linkage_path="sampleRelationships_to_samples_object")</t>
+  </si>
+  <si>
+    <t>organizations</t>
+  </si>
+  <si>
+    <t>""</t>
+  </si>
+  <si>
+    <t>addressID</t>
   </si>
 </sst>
 </file>
@@ -461,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BB192A8-54D6-B94E-B895-8C1E220F8CDD}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
@@ -525,6 +534,17 @@
         <v>12</v>
       </c>
     </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
General PHA4GE to ODM v2 ID code changes
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
+++ b/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/pha4ge-to-v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F2A4F17-3875-D64D-B39A-93BB33B1F810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{226CB708-A1B4-A84D-B2C7-39F9E019002E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{7D7FC1CC-FEF0-9E4D-91AE-A58F443803E1}"/>
   </bookViews>
   <sheets>
-    <sheet name="sites" sheetId="1" r:id="rId1"/>
+    <sheet name="id_code" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>

<commit_message>
Add ID code for protocolRelationships table
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
+++ b/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/pha4ge-to-v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{226CB708-A1B4-A84D-B2C7-39F9E019002E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{880BFD07-8C06-1649-8C3D-E692A9C14810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{7D7FC1CC-FEF0-9E4D-91AE-A58F443803E1}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
   <si>
     <t>sites</t>
   </si>
@@ -107,6 +107,27 @@
   </si>
   <si>
     <t>addressID</t>
+  </si>
+  <si>
+    <t>protocolRelationships</t>
+  </si>
+  <si>
+    <t>stepIDObj</t>
+  </si>
+  <si>
+    <t>dat.protocolSteps.get_first_linked_value("stepID", linkage_path="protocolRelationships_to_protocolSteps_subject")</t>
+  </si>
+  <si>
+    <t>dat.protocolSteps.get_first_linked_value("stepID", linkage_path="protocolRelationships_to_protocolSteps_object")</t>
+  </si>
+  <si>
+    <t>stepIDSub</t>
+  </si>
+  <si>
+    <t>protocolIDContainer</t>
+  </si>
+  <si>
+    <t>dat.protocols.get_first_linked_value("protocolID", linkage_path="protocolRelationships_to_protocols_container")</t>
   </si>
 </sst>
 </file>
@@ -470,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BB192A8-54D6-B94E-B895-8C1E220F8CDD}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
@@ -545,6 +566,39 @@
         <v>14</v>
       </c>
     </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
Remove comments for accessions.measureSetRepID
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
+++ b/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/pha4ge-to-v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85144BDB-C3E9-0343-911D-354151AAC5AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DFFC1AF-837B-5543-9020-D87E9D95B93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{7D7FC1CC-FEF0-9E4D-91AE-A58F443803E1}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
   <si>
     <t>sites</t>
   </si>
@@ -139,9 +139,6 @@
     <t>measureRepID</t>
   </si>
   <si>
-    <t>accession should link to measureRepID for detLinClade first, if no detLinClade then link with the only measureSetRepID</t>
-  </si>
-  <si>
     <t>organizationID</t>
   </si>
   <si>
@@ -149,9 +146,6 @@
   </si>
   <si>
     <t>dat.measures.get_first_linked_value("measureRepID", linkage_path="accessions_to_measures_measureRepID")</t>
-  </si>
-  <si>
-    <t>target = "" if dat.accessions.measureRepID else dat.measureSets.measureSetRepID</t>
   </si>
   <si>
     <t>"" if dat.accessions.measureRepID else dat.measureSets.measureSetRepID</t>
@@ -634,14 +628,9 @@
         <v>24</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D14" t="s">
-        <v>30</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>26</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -651,7 +640,7 @@
         <v>25</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -659,10 +648,10 @@
         <v>23</v>
       </c>
       <c r="B16" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" t="s">
         <v>27</v>
-      </c>
-      <c r="C16" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixes to sites.sampleShed and sites.siteType ID code to properly handle multivalued values.
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
+++ b/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/pha4ge-to-v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DFFC1AF-837B-5543-9020-D87E9D95B93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A53ADDFC-639F-EB43-B438-EA57717D7575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{7D7FC1CC-FEF0-9E4D-91AE-A58F443803E1}"/>
   </bookViews>
@@ -55,100 +55,126 @@
     <t>siteType</t>
   </si>
   <si>
-    <t>def get_sample_shed_type(check_first, check_with_prefix, prefix):
-    if check_first is not None and len(str(check_first)) &gt; 0:
-        if not isinstance(check_first, list):
-            check_first = [check_first]
-        for cur in check_first:
-            if cur and len(cur) &gt; 0:
-                return cur
-    for val in check_with_prefix:
-        if str(val).startswith(prefix):
-            return str(val).split(prefix, maxsplit=1)[1]
-    return ''        
+    <t>sampleRelationships</t>
+  </si>
+  <si>
+    <t>sampleIDSubject</t>
+  </si>
+  <si>
+    <t>sampleIDObject</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("sampleID", linkage_path="sampleRelationships_to_samples_subject")</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("sampleID", linkage_path="sampleRelationships_to_samples_object")</t>
+  </si>
+  <si>
+    <t>organizations</t>
+  </si>
+  <si>
+    <t>""</t>
+  </si>
+  <si>
+    <t>addressID</t>
+  </si>
+  <si>
+    <t>protocolRelationships</t>
+  </si>
+  <si>
+    <t>stepIDObj</t>
+  </si>
+  <si>
+    <t>dat.protocolSteps.get_first_linked_value("stepID", linkage_path="protocolRelationships_to_protocolSteps_subject")</t>
+  </si>
+  <si>
+    <t>dat.protocolSteps.get_first_linked_value("stepID", linkage_path="protocolRelationships_to_protocolSteps_object")</t>
+  </si>
+  <si>
+    <t>stepIDSub</t>
+  </si>
+  <si>
+    <t>protocolIDContainer</t>
+  </si>
+  <si>
+    <t>dat.protocols.get_first_linked_value("protocolID", linkage_path="protocolRelationships_to_protocols_container")</t>
+  </si>
+  <si>
+    <t>accessions</t>
+  </si>
+  <si>
+    <t>measureSetRepID</t>
+  </si>
+  <si>
+    <t>measureRepID</t>
+  </si>
+  <si>
+    <t>organizationID</t>
+  </si>
+  <si>
+    <t>dat.organizations.organizationID</t>
+  </si>
+  <si>
+    <t>dat.measures.get_first_linked_value("measureRepID", linkage_path="accessions_to_measures_measureRepID")</t>
+  </si>
+  <si>
+    <t>"" if dat.accessions.measureRepID else dat.measureSets.measureSetRepID</t>
+  </si>
+  <si>
+    <t>def select_from(values, prefix):
+    multivalued = isinstance(values, (list, tuple))
+    if not multivalued:
+        values = [values]
+    results = []
+    # Iterate over all values, find non-empty values that start with prefix
+    # If prefix is empty then any  non-empty string matches
+    for cur in values:
+        if cur and len(cur) &gt; 0:
+            if prefix and str(cur).startswith(prefix):
+                results.append(str(cur).split(prefix, maxsplit=1)[1])
+            elif not prefix:
+                results.append(cur)
+    if not multivalued and len(results) &gt; 0:
+        results = results[0]
+    return results if results else ''
+def get_sample_shed_type(check_first, check_with_prefix, prefix):
+    results = select_from(check_first, '')
+    if results:
+        return results
+    results = select_from(check_with_prefix, prefix)
+    if results:
+        return results
+    return ''
 #target = get_sample_shed_type(dat.sites.__siteType, dat.sites.__sampleShed, 'siteType:')
 target = get_sample_shed_type(None, dat.sites.__sampleShed, 'sampleShed:')</t>
   </si>
   <si>
-    <t>def get_sample_shed_type(check_first, check_with_prefix, prefix):
-    if check_first is not None and len(str(check_first)) &gt; 0:
-        if not isinstance(check_first, list):
-            check_first = [check_first]
-        for cur in check_first:
-            if cur and len(cur) &gt; 0:
-                return cur
-    for val in check_with_prefix:
-        if str(val).startswith(prefix):
-            return str(val).split(prefix, maxsplit=1)[1]
-    return ''        
+    <t>def select_from(values, prefix):
+    multivalued = isinstance(values, (list, tuple))
+    if not multivalued:
+        values = [values]
+    results = []
+    # Iterate over all values, find non-empty values that start with prefix
+    # If prefix is empty then any  non-empty string matches
+    for cur in values:
+        if cur and len(cur) &gt; 0:
+            if prefix and str(cur).startswith(prefix):
+                results.append(str(cur).split(prefix, maxsplit=1)[1])
+            elif not prefix:
+                results.append(cur)
+    if not multivalued and len(results) &gt; 0:
+        results = results[0]
+    return results if results else ''
+def get_sample_shed_type(check_first, check_with_prefix, prefix):
+    results = select_from(check_first, '')
+    if results:
+        return results
+    results = select_from(check_with_prefix, prefix)
+    if results:
+        return results
+    return ''
 target = get_sample_shed_type(dat.sites.__siteType, dat.sites.__sampleShed, 'siteType:')
 #target = get_sample_shed_type(None, dat.sites.__sampleShed, 'sampleShed:')</t>
-  </si>
-  <si>
-    <t>sampleRelationships</t>
-  </si>
-  <si>
-    <t>sampleIDSubject</t>
-  </si>
-  <si>
-    <t>sampleIDObject</t>
-  </si>
-  <si>
-    <t>dat.samples.get_first_linked_value("sampleID", linkage_path="sampleRelationships_to_samples_subject")</t>
-  </si>
-  <si>
-    <t>dat.samples.get_first_linked_value("sampleID", linkage_path="sampleRelationships_to_samples_object")</t>
-  </si>
-  <si>
-    <t>organizations</t>
-  </si>
-  <si>
-    <t>""</t>
-  </si>
-  <si>
-    <t>addressID</t>
-  </si>
-  <si>
-    <t>protocolRelationships</t>
-  </si>
-  <si>
-    <t>stepIDObj</t>
-  </si>
-  <si>
-    <t>dat.protocolSteps.get_first_linked_value("stepID", linkage_path="protocolRelationships_to_protocolSteps_subject")</t>
-  </si>
-  <si>
-    <t>dat.protocolSteps.get_first_linked_value("stepID", linkage_path="protocolRelationships_to_protocolSteps_object")</t>
-  </si>
-  <si>
-    <t>stepIDSub</t>
-  </si>
-  <si>
-    <t>protocolIDContainer</t>
-  </si>
-  <si>
-    <t>dat.protocols.get_first_linked_value("protocolID", linkage_path="protocolRelationships_to_protocols_container")</t>
-  </si>
-  <si>
-    <t>accessions</t>
-  </si>
-  <si>
-    <t>measureSetRepID</t>
-  </si>
-  <si>
-    <t>measureRepID</t>
-  </si>
-  <si>
-    <t>organizationID</t>
-  </si>
-  <si>
-    <t>dat.organizations.organizationID</t>
-  </si>
-  <si>
-    <t>dat.measures.get_first_linked_value("measureRepID", linkage_path="accessions_to_measures_measureRepID")</t>
-  </si>
-  <si>
-    <t>"" if dat.accessions.measureRepID else dat.measureSets.measureSetRepID</t>
   </si>
 </sst>
 </file>
@@ -532,7 +558,7 @@
       </c>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="1:6" ht="356" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -540,10 +566,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="272" x14ac:dyDescent="0.2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -551,107 +577,107 @@
         <v>5</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>7</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
         <v>9</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>10</v>
-      </c>
-      <c r="C6" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
         <v>13</v>
       </c>
-      <c r="B8" t="s">
-        <v>15</v>
-      </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" t="s">
         <v>16</v>
-      </c>
-      <c r="B10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" t="s">
         <v>17</v>
-      </c>
-      <c r="C11" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" t="s">
         <v>23</v>
       </c>
-      <c r="B15" t="s">
-        <v>25</v>
-      </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C16" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updates to ODM v2/v3 ID code for PHA4GE to ODM v2/v3 mapping
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
+++ b/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/pha4ge-to-v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{413DD3B4-6F81-2544-B198-04293F589335}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04AF32E4-7D0F-0546-BCEE-9B0AC3B4C70B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{7D7FC1CC-FEF0-9E4D-91AE-A58F443803E1}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
   <si>
     <t>sites</t>
   </si>
@@ -107,12 +107,6 @@
   </si>
   <si>
     <t>measureRepID</t>
-  </si>
-  <si>
-    <t>organizationID</t>
-  </si>
-  <si>
-    <t>dat.organizations.organizationID</t>
   </si>
   <si>
     <t>dat.measures.get_first_linked_value("measureRepID", linkage_path="accessions_to_measures_measureRepID")</t>
@@ -175,6 +169,27 @@
     return ''
 target = get_sample_shed_type(dat.sites.__siteType, dat.sites.__sampleShed, 'siteType:')
 #target = get_sample_shed_type(None, dat.sites.__sampleShed, 'sampleShed:')</t>
+  </si>
+  <si>
+    <t>qualityReports</t>
+  </si>
+  <si>
+    <t>dat.measures.get_first_linked_value("measureRepID", linkage_path="qualityReports_to_measures_measure")</t>
+  </si>
+  <si>
+    <t>datasets</t>
+  </si>
+  <si>
+    <t>funderCont</t>
+  </si>
+  <si>
+    <t>dat.contacts.get_first_linked_value("contactID", linkage_path="datasets_to_contacts_funderCont_contactID")</t>
+  </si>
+  <si>
+    <t>custodyCont</t>
+  </si>
+  <si>
+    <t>dat.contacts.get_first_linked_value("contactID", linkage_path="datasets_to_contacts_custodyCont_contactID")</t>
   </si>
 </sst>
 </file>
@@ -538,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BB192A8-54D6-B94E-B895-8C1E220F8CDD}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
@@ -558,7 +573,7 @@
       </c>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -566,10 +581,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -577,7 +592,7 @@
         <v>5</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -654,7 +669,7 @@
         <v>22</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F14" s="1"/>
     </row>
@@ -666,18 +681,40 @@
         <v>23</v>
       </c>
       <c r="C15" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" t="s">
         <v>24</v>
       </c>
-      <c r="C16" t="s">
-        <v>25</v>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" t="s">
+        <v>31</v>
+      </c>
+      <c r="C19" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added ID code for extra biological/technical replicate rows in samples table, and entries in sampleRelationships table
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
+++ b/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/pha4ge-to-v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04AF32E4-7D0F-0546-BCEE-9B0AC3B4C70B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F0120D7-86A9-1446-B4E1-9EE38FEA3EB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{7D7FC1CC-FEF0-9E4D-91AE-A58F443803E1}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="97">
   <si>
     <t>sites</t>
   </si>
@@ -190,6 +190,192 @@
   </si>
   <si>
     <t>dat.contacts.get_first_linked_value("contactID", linkage_path="datasets_to_contacts_custodyCont_contactID")</t>
+  </si>
+  <si>
+    <t>samples</t>
+  </si>
+  <si>
+    <t>sampleID:replicate</t>
+  </si>
+  <si>
+    <t>protocolID:replicate</t>
+  </si>
+  <si>
+    <t>organizationID:replicate</t>
+  </si>
+  <si>
+    <t>contactID:replicate</t>
+  </si>
+  <si>
+    <t>siteID:replicate</t>
+  </si>
+  <si>
+    <t>purpose:replicate</t>
+  </si>
+  <si>
+    <t>saMaterial:replicate</t>
+  </si>
+  <si>
+    <t>datasetID:replicate</t>
+  </si>
+  <si>
+    <t>origin:replicate</t>
+  </si>
+  <si>
+    <t>repType:replicate</t>
+  </si>
+  <si>
+    <t>collType:replicate</t>
+  </si>
+  <si>
+    <t>collPer:replicate</t>
+  </si>
+  <si>
+    <t>collNum:replicate</t>
+  </si>
+  <si>
+    <t>pooled:replicate</t>
+  </si>
+  <si>
+    <t>collDT:replicate</t>
+  </si>
+  <si>
+    <t>collDTStart:replicate</t>
+  </si>
+  <si>
+    <t>collDTEnd:replicate</t>
+  </si>
+  <si>
+    <t>collDate:replicate</t>
+  </si>
+  <si>
+    <t>collAppxT:replicate</t>
+  </si>
+  <si>
+    <t>epiWeekStart:replicate</t>
+  </si>
+  <si>
+    <t>epiWeek:replicate</t>
+  </si>
+  <si>
+    <t>epiYear:replicate</t>
+  </si>
+  <si>
+    <t>sentDate:replicate</t>
+  </si>
+  <si>
+    <t>recDate:replicate</t>
+  </si>
+  <si>
+    <t>reportable:replicate</t>
+  </si>
+  <si>
+    <t>lastEdited:replicate</t>
+  </si>
+  <si>
+    <t>notes:replicate</t>
+  </si>
+  <si>
+    <t>dat.samples.__repType</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.samples.get_first_linked_value("sampleID", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True), dat.samples.__sampleID)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("protocolID", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("organizationID", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("contactID", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("siteID", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("purpose", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("saMaterial", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("datasetID", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("origin", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("collType", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("collPer", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("collNum", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("pooled", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("collDT", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("collDTStart", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("collDTEnd", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("collDate", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("collAppxT", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("epiWeekStart", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("epiWeek", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("epiYear", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("sentDate", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("recDate", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("reportable", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("lastEdited", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("notes", linkage_path="samples_to_samples_replicate_pairing", ignore_current_row=True)</t>
+  </si>
+  <si>
+    <t>dat.samples.get_first_linked_value("sampleID", linkage_path="sampleRelationships_to_samples_object_replicate")</t>
+  </si>
+  <si>
+    <t>sampleIDObject:replicate</t>
+  </si>
+  <si>
+    <t>sampleIDSubject:replicate</t>
+  </si>
+  <si>
+    <t>fn.makeid(dat.sampleRelationships.__sampleRelationshipsID)</t>
+  </si>
+  <si>
+    <t>fn.makeid("rel")</t>
+  </si>
+  <si>
+    <t>code1</t>
+  </si>
+  <si>
+    <t>sampleRelationshipsID:replicate</t>
   </si>
 </sst>
 </file>
@@ -553,11 +739,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BB192A8-54D6-B94E-B895-8C1E220F8CDD}">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="98.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -571,50 +757,53 @@
       <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1"/>
-    </row>
-    <row r="2" spans="1:6" ht="409.5" x14ac:dyDescent="0.2">
+      <c r="D1" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="409.5" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+      <c r="F2" s="1"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -661,60 +850,392 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F14" s="1"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" t="s">
         <v>23</v>
       </c>
-      <c r="C15" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="409.5" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="B17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C17" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="C19" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>33</v>
+        <v>8</v>
       </c>
       <c r="C20" t="s">
-        <v>34</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" t="s">
+        <v>92</v>
+      </c>
+      <c r="C21" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" t="s">
+        <v>91</v>
+      </c>
+      <c r="C22" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23" t="s">
+        <v>96</v>
+      </c>
+      <c r="C23" t="s">
+        <v>93</v>
+      </c>
+      <c r="D23" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" t="s">
+        <v>36</v>
+      </c>
+      <c r="C25" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" t="s">
+        <v>37</v>
+      </c>
+      <c r="C26" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>35</v>
+      </c>
+      <c r="B27" t="s">
+        <v>38</v>
+      </c>
+      <c r="C27" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" t="s">
+        <v>39</v>
+      </c>
+      <c r="C28" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29" t="s">
+        <v>40</v>
+      </c>
+      <c r="C29" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" t="s">
+        <v>41</v>
+      </c>
+      <c r="C30" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>35</v>
+      </c>
+      <c r="B31" t="s">
+        <v>42</v>
+      </c>
+      <c r="C31" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>35</v>
+      </c>
+      <c r="B32" t="s">
+        <v>43</v>
+      </c>
+      <c r="C32" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" t="s">
+        <v>44</v>
+      </c>
+      <c r="C33" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>35</v>
+      </c>
+      <c r="B34" t="s">
+        <v>45</v>
+      </c>
+      <c r="C34" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35" t="s">
+        <v>46</v>
+      </c>
+      <c r="C35" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>47</v>
+      </c>
+      <c r="C36" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>35</v>
+      </c>
+      <c r="B37" t="s">
+        <v>48</v>
+      </c>
+      <c r="C37" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>35</v>
+      </c>
+      <c r="B38" t="s">
+        <v>49</v>
+      </c>
+      <c r="C38" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39" t="s">
+        <v>50</v>
+      </c>
+      <c r="C39" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>35</v>
+      </c>
+      <c r="B40" t="s">
+        <v>51</v>
+      </c>
+      <c r="C40" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>35</v>
+      </c>
+      <c r="B41" t="s">
+        <v>52</v>
+      </c>
+      <c r="C41" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>35</v>
+      </c>
+      <c r="B42" t="s">
+        <v>53</v>
+      </c>
+      <c r="C42" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>35</v>
+      </c>
+      <c r="B43" t="s">
+        <v>54</v>
+      </c>
+      <c r="C43" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>35</v>
+      </c>
+      <c r="B44" t="s">
+        <v>55</v>
+      </c>
+      <c r="C44" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>35</v>
+      </c>
+      <c r="B45" t="s">
+        <v>56</v>
+      </c>
+      <c r="C45" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>35</v>
+      </c>
+      <c r="B46" t="s">
+        <v>57</v>
+      </c>
+      <c r="C46" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>35</v>
+      </c>
+      <c r="B47" t="s">
+        <v>58</v>
+      </c>
+      <c r="C47" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>35</v>
+      </c>
+      <c r="B48" t="s">
+        <v>59</v>
+      </c>
+      <c r="C48" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>35</v>
+      </c>
+      <c r="B49" t="s">
+        <v>60</v>
+      </c>
+      <c r="C49" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>35</v>
+      </c>
+      <c r="B50" t="s">
+        <v>61</v>
+      </c>
+      <c r="C50" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>35</v>
+      </c>
+      <c r="B51" t="s">
+        <v>62</v>
+      </c>
+      <c r="C51" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Pass all primary key IDs to fn.makeid
</commit_message>
<xml_diff>
--- a/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
+++ b/odm_map/data/modules/pha4ge-to-v2/ids/pha4ge_to_v2_id_code.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-Mapper/PHES-ODM-Mapper/odm_map/data/modules/pha4ge-to-v2/ids/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C88DFE0-8842-904B-B015-F7DF8CC63EC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09774564-3719-2742-8139-54B4EDE4D6CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="40960" windowHeight="20900" xr2:uid="{7D7FC1CC-FEF0-9E4D-91AE-A58F443803E1}"/>
   </bookViews>
@@ -366,16 +366,16 @@
     <t>sampleIDSubject:replicate</t>
   </si>
   <si>
-    <t>fn.makeid("rel")</t>
-  </si>
-  <si>
     <t>code1</t>
   </si>
   <si>
     <t>sampleRelationshipsID:replicate</t>
   </si>
   <si>
-    <t>dat.sampleRelationships.__sampleRelationshipsID</t>
+    <t>fn.makeid(dat.sampleRelationships.__sampleRelationshipsID)</t>
+  </si>
+  <si>
+    <t>fn.makeid("sar")</t>
   </si>
 </sst>
 </file>
@@ -758,7 +758,7 @@
         <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -932,13 +932,13 @@
         <v>6</v>
       </c>
       <c r="B23" t="s">
+        <v>94</v>
+      </c>
+      <c r="C23" t="s">
         <v>95</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>96</v>
-      </c>
-      <c r="D23" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>